<commit_message>
docs(deliverables): update university thesis status reports and WBS documentation
- Add Week 05 and Week 06 status reports
- Update Project Charter, SOW, and WBS benchmarking deliverables
</commit_message>
<xml_diff>
--- a/docs_ute/(2) FocusFlow-Work-Breakdown-Structure-with-Gantt-Chart.xlsx
+++ b/docs_ute/(2) FocusFlow-Work-Breakdown-Structure-with-Gantt-Chart.xlsx
@@ -217,10 +217,10 @@
     <t>Thiết lập nền tảng &amp; Module cơ sở (Project Setup &amp; Foundation Modules)</t>
   </si>
   <si>
-    <t>Khởi tạo Repository, cấu hình dự án &amp; Thiết lập CI/CD Pipeline tự động</t>
+    <t>Khởi tạo Repository, cấu hình dự án, Alembic Database Migrations &amp; Thiết lập CI/CD Pipeline tự động</t>
   </si>
   <si>
-    <t>Xây dựng Module Xác thực &amp; Hồ sơ người dùng (FR-AUTH: JWT, Session Guard)</t>
+    <t>Xây dựng Module Xác thực, Phân quyền RBAC (User/Admin) &amp; Hồ sơ người dùng (FR-AUTH)</t>
   </si>
   <si>
     <t>Xây dựng Module Cấu hình thời gian rảnh lai (FR-AVAIL Mode A Quota &amp; Mode B)</t>
@@ -247,7 +247,7 @@
     <t>Xử lý gián đoạn phiên học &amp; Hoàn trả task dở dang về Backlog</t>
   </si>
   <si>
-    <t>Phát triển thuật toán thích ứng quá hạn tất định (Deterministic Overdue Shift)</t>
+    <t>Phát triển thuật toán thích ứng quá hạn tất định &amp; Celery Beat Scheduled Tasks (FR-OVERDUE)</t>
   </si>
   <si>
     <t>Phát triển tính năng Tạm dừng lộ trình (Pause Roadmap &amp; Domino Shift)</t>
@@ -265,7 +265,7 @@
     <t>Tích hợp AI Review phân tích định tính từ số liệu thống kê &amp; Key Takeaways</t>
   </si>
   <si>
-    <t>Xây dựng Service-level Quota Guard Middleware &amp; Mock Upgrade Sandbox</t>
+    <t>Xây dựng Service-level Quota Guard, Admin Quota Override &amp; Mock Upgrade Sandbox</t>
   </si>
   <si>
     <t>Kiểm thử phần mềm &amp; Đo lường NFRs (Software Testing &amp; NFR Verification)</t>
@@ -1065,7 +1065,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="15.0" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.22" customWidth="1"/>
@@ -1819,141 +1819,141 @@
       <c r="H7" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="I7" s="23" t="s">
+      <c r="I7" s="52" t="s">
         <v>21</v>
       </c>
-      <c r="J7" s="24"/>
-      <c r="K7" s="24"/>
-      <c r="L7" s="24"/>
-      <c r="M7" s="24"/>
-      <c r="N7" s="24"/>
-      <c r="O7" s="25"/>
-      <c r="P7" s="23" t="s">
+      <c r="J7" s="52"/>
+      <c r="K7" s="52"/>
+      <c r="L7" s="52"/>
+      <c r="M7" s="52"/>
+      <c r="N7" s="52"/>
+      <c r="O7" s="52"/>
+      <c r="P7" s="52" t="s">
         <v>22</v>
       </c>
-      <c r="Q7" s="24"/>
-      <c r="R7" s="24"/>
-      <c r="S7" s="24"/>
-      <c r="T7" s="24"/>
-      <c r="U7" s="24"/>
-      <c r="V7" s="25"/>
-      <c r="W7" s="23" t="s">
+      <c r="Q7" s="52"/>
+      <c r="R7" s="52"/>
+      <c r="S7" s="52"/>
+      <c r="T7" s="52"/>
+      <c r="U7" s="52"/>
+      <c r="V7" s="52"/>
+      <c r="W7" s="52" t="s">
         <v>23</v>
       </c>
-      <c r="X7" s="24"/>
-      <c r="Y7" s="24"/>
-      <c r="Z7" s="24"/>
-      <c r="AA7" s="24"/>
-      <c r="AB7" s="24"/>
-      <c r="AC7" s="25"/>
-      <c r="AD7" s="23" t="s">
+      <c r="X7" s="52"/>
+      <c r="Y7" s="52"/>
+      <c r="Z7" s="52"/>
+      <c r="AA7" s="52"/>
+      <c r="AB7" s="52"/>
+      <c r="AC7" s="52"/>
+      <c r="AD7" s="52" t="s">
         <v>24</v>
       </c>
-      <c r="AE7" s="24"/>
-      <c r="AF7" s="24"/>
-      <c r="AG7" s="24"/>
-      <c r="AH7" s="24"/>
-      <c r="AI7" s="24"/>
-      <c r="AJ7" s="25"/>
-      <c r="AK7" s="23" t="s">
+      <c r="AE7" s="52"/>
+      <c r="AF7" s="52"/>
+      <c r="AG7" s="52"/>
+      <c r="AH7" s="52"/>
+      <c r="AI7" s="52"/>
+      <c r="AJ7" s="52"/>
+      <c r="AK7" s="52" t="s">
         <v>25</v>
       </c>
-      <c r="AL7" s="24"/>
-      <c r="AM7" s="24"/>
-      <c r="AN7" s="24"/>
-      <c r="AO7" s="24"/>
-      <c r="AP7" s="24"/>
-      <c r="AQ7" s="25"/>
-      <c r="AR7" s="23" t="s">
+      <c r="AL7" s="52"/>
+      <c r="AM7" s="52"/>
+      <c r="AN7" s="52"/>
+      <c r="AO7" s="52"/>
+      <c r="AP7" s="52"/>
+      <c r="AQ7" s="52"/>
+      <c r="AR7" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="AS7" s="24"/>
-      <c r="AT7" s="24"/>
-      <c r="AU7" s="24"/>
-      <c r="AV7" s="24"/>
-      <c r="AW7" s="24"/>
-      <c r="AX7" s="25"/>
-      <c r="AY7" s="23" t="s">
+      <c r="AS7" s="52"/>
+      <c r="AT7" s="52"/>
+      <c r="AU7" s="52"/>
+      <c r="AV7" s="52"/>
+      <c r="AW7" s="52"/>
+      <c r="AX7" s="52"/>
+      <c r="AY7" s="52" t="s">
         <v>27</v>
       </c>
-      <c r="AZ7" s="24"/>
-      <c r="BA7" s="24"/>
-      <c r="BB7" s="24"/>
-      <c r="BC7" s="24"/>
-      <c r="BD7" s="24"/>
-      <c r="BE7" s="25"/>
-      <c r="BF7" s="23" t="s">
+      <c r="AZ7" s="52"/>
+      <c r="BA7" s="52"/>
+      <c r="BB7" s="52"/>
+      <c r="BC7" s="52"/>
+      <c r="BD7" s="52"/>
+      <c r="BE7" s="52"/>
+      <c r="BF7" s="52" t="s">
         <v>28</v>
       </c>
-      <c r="BG7" s="24"/>
-      <c r="BH7" s="24"/>
-      <c r="BI7" s="24"/>
-      <c r="BJ7" s="24"/>
-      <c r="BK7" s="24"/>
-      <c r="BL7" s="25"/>
-      <c r="BM7" s="23" t="s">
+      <c r="BG7" s="52"/>
+      <c r="BH7" s="52"/>
+      <c r="BI7" s="52"/>
+      <c r="BJ7" s="52"/>
+      <c r="BK7" s="52"/>
+      <c r="BL7" s="52"/>
+      <c r="BM7" s="52" t="s">
         <v>29</v>
       </c>
-      <c r="BN7" s="24"/>
-      <c r="BO7" s="24"/>
-      <c r="BP7" s="24"/>
-      <c r="BQ7" s="24"/>
-      <c r="BR7" s="24"/>
-      <c r="BS7" s="25"/>
-      <c r="BT7" s="23" t="s">
+      <c r="BN7" s="52"/>
+      <c r="BO7" s="52"/>
+      <c r="BP7" s="52"/>
+      <c r="BQ7" s="52"/>
+      <c r="BR7" s="52"/>
+      <c r="BS7" s="52"/>
+      <c r="BT7" s="52" t="s">
         <v>30</v>
       </c>
-      <c r="BU7" s="24"/>
-      <c r="BV7" s="24"/>
-      <c r="BW7" s="24"/>
-      <c r="BX7" s="24"/>
-      <c r="BY7" s="24"/>
-      <c r="BZ7" s="25"/>
-      <c r="CA7" s="23" t="s">
+      <c r="BU7" s="52"/>
+      <c r="BV7" s="52"/>
+      <c r="BW7" s="52"/>
+      <c r="BX7" s="52"/>
+      <c r="BY7" s="52"/>
+      <c r="BZ7" s="52"/>
+      <c r="CA7" s="52" t="s">
         <v>31</v>
       </c>
-      <c r="CB7" s="24"/>
-      <c r="CC7" s="24"/>
-      <c r="CD7" s="24"/>
-      <c r="CE7" s="24"/>
-      <c r="CF7" s="24"/>
-      <c r="CG7" s="25"/>
-      <c r="CH7" s="23" t="s">
+      <c r="CB7" s="52"/>
+      <c r="CC7" s="52"/>
+      <c r="CD7" s="52"/>
+      <c r="CE7" s="52"/>
+      <c r="CF7" s="52"/>
+      <c r="CG7" s="52"/>
+      <c r="CH7" s="52" t="s">
         <v>32</v>
       </c>
-      <c r="CI7" s="24"/>
-      <c r="CJ7" s="24"/>
-      <c r="CK7" s="24"/>
-      <c r="CL7" s="24"/>
-      <c r="CM7" s="24"/>
-      <c r="CN7" s="25"/>
-      <c r="CO7" s="23" t="s">
+      <c r="CI7" s="52"/>
+      <c r="CJ7" s="52"/>
+      <c r="CK7" s="52"/>
+      <c r="CL7" s="52"/>
+      <c r="CM7" s="52"/>
+      <c r="CN7" s="52"/>
+      <c r="CO7" s="52" t="s">
         <v>33</v>
       </c>
-      <c r="CP7" s="24"/>
-      <c r="CQ7" s="24"/>
-      <c r="CR7" s="24"/>
-      <c r="CS7" s="24"/>
-      <c r="CT7" s="24"/>
-      <c r="CU7" s="25"/>
-      <c r="CV7" s="23" t="s">
+      <c r="CP7" s="52"/>
+      <c r="CQ7" s="52"/>
+      <c r="CR7" s="52"/>
+      <c r="CS7" s="52"/>
+      <c r="CT7" s="52"/>
+      <c r="CU7" s="52"/>
+      <c r="CV7" s="52" t="s">
         <v>34</v>
       </c>
-      <c r="CW7" s="24"/>
-      <c r="CX7" s="24"/>
-      <c r="CY7" s="24"/>
-      <c r="CZ7" s="24"/>
-      <c r="DA7" s="24"/>
-      <c r="DB7" s="25"/>
-      <c r="DC7" s="23" t="s">
+      <c r="CW7" s="52"/>
+      <c r="CX7" s="52"/>
+      <c r="CY7" s="52"/>
+      <c r="CZ7" s="52"/>
+      <c r="DA7" s="52"/>
+      <c r="DB7" s="52"/>
+      <c r="DC7" s="52" t="s">
         <v>35</v>
       </c>
-      <c r="DD7" s="24"/>
-      <c r="DE7" s="24"/>
-      <c r="DF7" s="24"/>
-      <c r="DG7" s="24"/>
-      <c r="DH7" s="24"/>
-      <c r="DI7" s="25"/>
+      <c r="DD7" s="52"/>
+      <c r="DE7" s="52"/>
+      <c r="DF7" s="52"/>
+      <c r="DG7" s="52"/>
+      <c r="DH7" s="52"/>
+      <c r="DI7" s="52"/>
     </row>
     <row r="8" ht="18.0" customHeight="1">
       <c r="A8" s="4"/>
@@ -2289,10 +2289,18 @@
         <v>43</v>
       </c>
       <c r="D9" s="42"/>
-      <c r="E9" s="43"/>
-      <c r="F9" s="43"/>
-      <c r="G9" s="44"/>
-      <c r="H9" s="45"/>
+      <c r="E9" s="43">
+        <f>MIN(E10:E12)</f>
+      </c>
+      <c r="F9" s="43">
+        <f>MAX(F10:F12)</f>
+      </c>
+      <c r="G9" s="44">
+        <f>DAYS(F9,E9)+1</f>
+      </c>
+      <c r="H9" s="45">
+        <f>AVERAGE(H10:H12)</f>
+      </c>
       <c r="I9" s="46"/>
       <c r="J9" s="46"/>
       <c r="K9" s="46"/>
@@ -2423,12 +2431,12 @@
       <c r="H10" s="51">
         <v>1.00</v>
       </c>
-      <c r="I10" s="53"/>
-      <c r="J10" s="53"/>
-      <c r="K10" s="53"/>
-      <c r="L10" s="53"/>
-      <c r="M10" s="53"/>
-      <c r="N10" s="53"/>
+      <c r="I10" s="55"/>
+      <c r="J10" s="55"/>
+      <c r="K10" s="55"/>
+      <c r="L10" s="55"/>
+      <c r="M10" s="55"/>
+      <c r="N10" s="55"/>
       <c r="O10" s="52"/>
       <c r="P10" s="52"/>
       <c r="Q10" s="52"/>
@@ -2557,11 +2565,11 @@
       <c r="J11" s="52"/>
       <c r="K11" s="52"/>
       <c r="L11" s="52"/>
-      <c r="M11" s="53"/>
-      <c r="N11" s="53"/>
-      <c r="O11" s="53"/>
-      <c r="P11" s="53"/>
-      <c r="Q11" s="53"/>
+      <c r="M11" s="55"/>
+      <c r="N11" s="55"/>
+      <c r="O11" s="55"/>
+      <c r="P11" s="55"/>
+      <c r="Q11" s="55"/>
       <c r="R11" s="52"/>
       <c r="S11" s="52"/>
       <c r="T11" s="52"/>
@@ -2690,11 +2698,11 @@
       <c r="M12" s="52"/>
       <c r="N12" s="52"/>
       <c r="O12" s="52"/>
-      <c r="P12" s="53"/>
-      <c r="Q12" s="53"/>
-      <c r="R12" s="53"/>
-      <c r="S12" s="53"/>
-      <c r="T12" s="53"/>
+      <c r="P12" s="55"/>
+      <c r="Q12" s="55"/>
+      <c r="R12" s="55"/>
+      <c r="S12" s="55"/>
+      <c r="T12" s="55"/>
       <c r="U12" s="52"/>
       <c r="V12" s="52"/>
       <c r="W12" s="52"/>
@@ -2798,10 +2806,18 @@
         <v>49</v>
       </c>
       <c r="D13" s="42"/>
-      <c r="E13" s="43"/>
-      <c r="F13" s="43"/>
-      <c r="G13" s="44"/>
-      <c r="H13" s="45"/>
+      <c r="E13" s="43">
+        <f>MIN(E14:E17)</f>
+      </c>
+      <c r="F13" s="43">
+        <f>MAX(F14:F17)</f>
+      </c>
+      <c r="G13" s="44">
+        <f>DAYS(F13,E13)+1</f>
+      </c>
+      <c r="H13" s="45">
+        <f>AVERAGE(H14:H17)</f>
+      </c>
       <c r="I13" s="46"/>
       <c r="J13" s="46"/>
       <c r="K13" s="46"/>
@@ -2941,13 +2957,13 @@
       <c r="O14" s="52"/>
       <c r="P14" s="52"/>
       <c r="Q14" s="52"/>
-      <c r="R14" s="53"/>
-      <c r="S14" s="53"/>
-      <c r="T14" s="53"/>
-      <c r="U14" s="53"/>
-      <c r="V14" s="53"/>
-      <c r="W14" s="53"/>
-      <c r="X14" s="53"/>
+      <c r="R14" s="55"/>
+      <c r="S14" s="55"/>
+      <c r="T14" s="55"/>
+      <c r="U14" s="55"/>
+      <c r="V14" s="55"/>
+      <c r="W14" s="55"/>
+      <c r="X14" s="55"/>
       <c r="Y14" s="52"/>
       <c r="Z14" s="52"/>
       <c r="AA14" s="52"/>
@@ -3074,12 +3090,12 @@
       <c r="R15" s="52"/>
       <c r="S15" s="52"/>
       <c r="T15" s="52"/>
-      <c r="U15" s="53"/>
-      <c r="V15" s="53"/>
-      <c r="W15" s="53"/>
-      <c r="X15" s="53"/>
-      <c r="Y15" s="53"/>
-      <c r="Z15" s="53"/>
+      <c r="U15" s="55"/>
+      <c r="V15" s="55"/>
+      <c r="W15" s="55"/>
+      <c r="X15" s="55"/>
+      <c r="Y15" s="55"/>
+      <c r="Z15" s="55"/>
       <c r="AA15" s="52"/>
       <c r="AB15" s="52"/>
       <c r="AC15" s="52"/>
@@ -3207,11 +3223,11 @@
       <c r="U16" s="52"/>
       <c r="V16" s="52"/>
       <c r="W16" s="52"/>
-      <c r="X16" s="53"/>
-      <c r="Y16" s="53"/>
-      <c r="Z16" s="53"/>
-      <c r="AA16" s="53"/>
-      <c r="AB16" s="53"/>
+      <c r="X16" s="55"/>
+      <c r="Y16" s="55"/>
+      <c r="Z16" s="55"/>
+      <c r="AA16" s="55"/>
+      <c r="AB16" s="55"/>
       <c r="AC16" s="52"/>
       <c r="AD16" s="52"/>
       <c r="AE16" s="52"/>
@@ -3340,9 +3356,9 @@
       <c r="X17" s="52"/>
       <c r="Y17" s="52"/>
       <c r="Z17" s="52"/>
-      <c r="AA17" s="53"/>
-      <c r="AB17" s="53"/>
-      <c r="AC17" s="53"/>
+      <c r="AA17" s="55"/>
+      <c r="AB17" s="55"/>
+      <c r="AC17" s="55"/>
       <c r="AD17" s="52"/>
       <c r="AE17" s="52"/>
       <c r="AF17" s="52"/>
@@ -3437,10 +3453,18 @@
         <v>55</v>
       </c>
       <c r="D18" s="42"/>
-      <c r="E18" s="43"/>
-      <c r="F18" s="43"/>
-      <c r="G18" s="44"/>
-      <c r="H18" s="45"/>
+      <c r="E18" s="43">
+        <f>MIN(E19:E22)</f>
+      </c>
+      <c r="F18" s="43">
+        <f>MAX(F19:F22)</f>
+      </c>
+      <c r="G18" s="44">
+        <f>DAYS(F18,E18)+1</f>
+      </c>
+      <c r="H18" s="45">
+        <f>AVERAGE(H19:H22)</f>
+      </c>
       <c r="I18" s="46"/>
       <c r="J18" s="46"/>
       <c r="K18" s="46"/>
@@ -3569,7 +3593,7 @@
         <v>6</v>
       </c>
       <c r="H19" s="51">
-        <v>0.80</v>
+        <v>1.00</v>
       </c>
       <c r="I19" s="52"/>
       <c r="J19" s="52"/>
@@ -3699,7 +3723,7 @@
         <v>6</v>
       </c>
       <c r="H20" s="51">
-        <v>0.50</v>
+        <v>1.00</v>
       </c>
       <c r="I20" s="52"/>
       <c r="J20" s="52"/>
@@ -3829,7 +3853,7 @@
         <v>6</v>
       </c>
       <c r="H21" s="51">
-        <v>0.40</v>
+        <v>1.00</v>
       </c>
       <c r="I21" s="52"/>
       <c r="J21" s="52"/>
@@ -3959,7 +3983,7 @@
         <v>5</v>
       </c>
       <c r="H22" s="51">
-        <v>0.30</v>
+        <v>1.00</v>
       </c>
       <c r="I22" s="52"/>
       <c r="J22" s="52"/>
@@ -4076,10 +4100,18 @@
         <v>60</v>
       </c>
       <c r="D23" s="42"/>
-      <c r="E23" s="43"/>
-      <c r="F23" s="43"/>
-      <c r="G23" s="44"/>
-      <c r="H23" s="45"/>
+      <c r="E23" s="43">
+        <f>MIN(E24:E27)</f>
+      </c>
+      <c r="F23" s="43">
+        <f>MAX(F24:F27)</f>
+      </c>
+      <c r="G23" s="44">
+        <f>DAYS(F23,E23)+1</f>
+      </c>
+      <c r="H23" s="45">
+        <f>AVERAGE(H24:H27)</f>
+      </c>
       <c r="I23" s="46"/>
       <c r="J23" s="46"/>
       <c r="K23" s="46"/>
@@ -4208,7 +4240,7 @@
         <v>8</v>
       </c>
       <c r="H24" s="51">
-        <v>0.40</v>
+        <v>1.00</v>
       </c>
       <c r="I24" s="52"/>
       <c r="J24" s="52"/>
@@ -4338,7 +4370,7 @@
         <v>7</v>
       </c>
       <c r="H25" s="51">
-        <v>0.30</v>
+        <v>1.00</v>
       </c>
       <c r="I25" s="52"/>
       <c r="J25" s="52"/>
@@ -4468,7 +4500,7 @@
         <v>5</v>
       </c>
       <c r="H26" s="51">
-        <v>0.00</v>
+        <v>1.00</v>
       </c>
       <c r="I26" s="52"/>
       <c r="J26" s="52"/>
@@ -4598,7 +4630,7 @@
         <v>4</v>
       </c>
       <c r="H27" s="51">
-        <v>0.00</v>
+        <v>1.00</v>
       </c>
       <c r="I27" s="52"/>
       <c r="J27" s="52"/>
@@ -4715,10 +4747,18 @@
         <v>65</v>
       </c>
       <c r="D28" s="42"/>
-      <c r="E28" s="43"/>
-      <c r="F28" s="43"/>
-      <c r="G28" s="44"/>
-      <c r="H28" s="45"/>
+      <c r="E28" s="43">
+        <f>MIN(E29:E31)</f>
+      </c>
+      <c r="F28" s="43">
+        <f>MAX(F29:F31)</f>
+      </c>
+      <c r="G28" s="44">
+        <f>DAYS(F28,E28)+1</f>
+      </c>
+      <c r="H28" s="45">
+        <f>AVERAGE(H29:H31)</f>
+      </c>
       <c r="I28" s="46"/>
       <c r="J28" s="46"/>
       <c r="K28" s="46"/>
@@ -4847,7 +4887,7 @@
         <v>6</v>
       </c>
       <c r="H29" s="51">
-        <v>0.00</v>
+        <v>0.30</v>
       </c>
       <c r="I29" s="52"/>
       <c r="J29" s="52"/>
@@ -4891,12 +4931,12 @@
       <c r="AV29" s="52"/>
       <c r="AW29" s="52"/>
       <c r="AX29" s="52"/>
-      <c r="AY29" s="56"/>
-      <c r="AZ29" s="56"/>
-      <c r="BA29" s="56"/>
-      <c r="BB29" s="56"/>
-      <c r="BC29" s="56"/>
-      <c r="BD29" s="56"/>
+      <c r="AY29" s="55"/>
+      <c r="AZ29" s="55"/>
+      <c r="BA29" s="55"/>
+      <c r="BB29" s="55"/>
+      <c r="BC29" s="55"/>
+      <c r="BD29" s="55"/>
       <c r="BE29" s="52"/>
       <c r="BF29" s="52"/>
       <c r="BG29" s="52"/>
@@ -5024,13 +5064,13 @@
       <c r="AY30" s="52"/>
       <c r="AZ30" s="52"/>
       <c r="BA30" s="52"/>
-      <c r="BB30" s="56"/>
-      <c r="BC30" s="56"/>
-      <c r="BD30" s="56"/>
-      <c r="BE30" s="56"/>
-      <c r="BF30" s="56"/>
-      <c r="BG30" s="56"/>
-      <c r="BH30" s="56"/>
+      <c r="BB30" s="55"/>
+      <c r="BC30" s="55"/>
+      <c r="BD30" s="55"/>
+      <c r="BE30" s="55"/>
+      <c r="BF30" s="55"/>
+      <c r="BG30" s="55"/>
+      <c r="BH30" s="55"/>
       <c r="BI30" s="52"/>
       <c r="BJ30" s="52"/>
       <c r="BK30" s="52"/>
@@ -5158,13 +5198,13 @@
       <c r="BC31" s="52"/>
       <c r="BD31" s="52"/>
       <c r="BE31" s="52"/>
-      <c r="BF31" s="56"/>
-      <c r="BG31" s="56"/>
-      <c r="BH31" s="56"/>
-      <c r="BI31" s="56"/>
-      <c r="BJ31" s="56"/>
-      <c r="BK31" s="56"/>
-      <c r="BL31" s="56"/>
+      <c r="BF31" s="55"/>
+      <c r="BG31" s="55"/>
+      <c r="BH31" s="55"/>
+      <c r="BI31" s="55"/>
+      <c r="BJ31" s="55"/>
+      <c r="BK31" s="55"/>
+      <c r="BL31" s="55"/>
       <c r="BM31" s="52"/>
       <c r="BN31" s="52"/>
       <c r="BO31" s="52"/>
@@ -5224,10 +5264,18 @@
         <v>69</v>
       </c>
       <c r="D32" s="42"/>
-      <c r="E32" s="43"/>
-      <c r="F32" s="43"/>
-      <c r="G32" s="44"/>
-      <c r="H32" s="45"/>
+      <c r="E32" s="43">
+        <f>MIN(E33:E35)</f>
+      </c>
+      <c r="F32" s="43">
+        <f>MAX(F33:F35)</f>
+      </c>
+      <c r="G32" s="44">
+        <f>DAYS(F32,E32)+1</f>
+      </c>
+      <c r="H32" s="45">
+        <f>AVERAGE(H33:H35)</f>
+      </c>
       <c r="I32" s="46"/>
       <c r="J32" s="46"/>
       <c r="K32" s="46"/>
@@ -5410,14 +5458,14 @@
       <c r="BF33" s="52"/>
       <c r="BG33" s="52"/>
       <c r="BH33" s="52"/>
-      <c r="BI33" s="56"/>
-      <c r="BJ33" s="56"/>
-      <c r="BK33" s="56"/>
-      <c r="BL33" s="56"/>
-      <c r="BM33" s="56"/>
-      <c r="BN33" s="56"/>
-      <c r="BO33" s="56"/>
-      <c r="BP33" s="56"/>
+      <c r="BI33" s="55"/>
+      <c r="BJ33" s="55"/>
+      <c r="BK33" s="55"/>
+      <c r="BL33" s="55"/>
+      <c r="BM33" s="55"/>
+      <c r="BN33" s="55"/>
+      <c r="BO33" s="55"/>
+      <c r="BP33" s="55"/>
       <c r="BQ33" s="52"/>
       <c r="BR33" s="52"/>
       <c r="BS33" s="52"/>
@@ -5545,15 +5593,15 @@
       <c r="BK34" s="52"/>
       <c r="BL34" s="52"/>
       <c r="BM34" s="52"/>
-      <c r="BN34" s="56"/>
-      <c r="BO34" s="56"/>
-      <c r="BP34" s="56"/>
-      <c r="BQ34" s="56"/>
-      <c r="BR34" s="56"/>
-      <c r="BS34" s="56"/>
-      <c r="BT34" s="56"/>
-      <c r="BU34" s="56"/>
-      <c r="BV34" s="56"/>
+      <c r="BN34" s="55"/>
+      <c r="BO34" s="55"/>
+      <c r="BP34" s="55"/>
+      <c r="BQ34" s="55"/>
+      <c r="BR34" s="55"/>
+      <c r="BS34" s="55"/>
+      <c r="BT34" s="55"/>
+      <c r="BU34" s="55"/>
+      <c r="BV34" s="55"/>
       <c r="BW34" s="52"/>
       <c r="BX34" s="52"/>
       <c r="BY34" s="52"/>
@@ -5681,14 +5729,14 @@
       <c r="BQ35" s="52"/>
       <c r="BR35" s="52"/>
       <c r="BS35" s="52"/>
-      <c r="BT35" s="56"/>
-      <c r="BU35" s="56"/>
-      <c r="BV35" s="56"/>
-      <c r="BW35" s="56"/>
-      <c r="BX35" s="56"/>
-      <c r="BY35" s="56"/>
-      <c r="BZ35" s="56"/>
-      <c r="CA35" s="56"/>
+      <c r="BT35" s="55"/>
+      <c r="BU35" s="55"/>
+      <c r="BV35" s="55"/>
+      <c r="BW35" s="55"/>
+      <c r="BX35" s="55"/>
+      <c r="BY35" s="55"/>
+      <c r="BZ35" s="55"/>
+      <c r="CA35" s="55"/>
       <c r="CB35" s="52"/>
       <c r="CC35" s="52"/>
       <c r="CD35" s="52"/>
@@ -5733,10 +5781,18 @@
         <v>73</v>
       </c>
       <c r="D36" s="42"/>
-      <c r="E36" s="43"/>
-      <c r="F36" s="43"/>
-      <c r="G36" s="44"/>
-      <c r="H36" s="45"/>
+      <c r="E36" s="43">
+        <f>MIN(E37:E41)</f>
+      </c>
+      <c r="F36" s="43">
+        <f>MAX(F37:F41)</f>
+      </c>
+      <c r="G36" s="44">
+        <f>DAYS(F36,E36)+1</f>
+      </c>
+      <c r="H36" s="45">
+        <f>AVERAGE(H37:H41)</f>
+      </c>
       <c r="I36" s="46"/>
       <c r="J36" s="46"/>
       <c r="K36" s="46"/>
@@ -5926,15 +5982,15 @@
       <c r="BM37" s="52"/>
       <c r="BN37" s="52"/>
       <c r="BO37" s="52"/>
-      <c r="BP37" s="56"/>
-      <c r="BQ37" s="56"/>
-      <c r="BR37" s="56"/>
-      <c r="BS37" s="56"/>
-      <c r="BT37" s="56"/>
-      <c r="BU37" s="56"/>
-      <c r="BV37" s="56"/>
-      <c r="BW37" s="56"/>
-      <c r="BX37" s="56"/>
+      <c r="BP37" s="55"/>
+      <c r="BQ37" s="55"/>
+      <c r="BR37" s="55"/>
+      <c r="BS37" s="55"/>
+      <c r="BT37" s="55"/>
+      <c r="BU37" s="55"/>
+      <c r="BV37" s="55"/>
+      <c r="BW37" s="55"/>
+      <c r="BX37" s="55"/>
       <c r="BY37" s="52"/>
       <c r="BZ37" s="52"/>
       <c r="CA37" s="52"/>
@@ -6062,12 +6118,12 @@
       <c r="BS38" s="52"/>
       <c r="BT38" s="52"/>
       <c r="BU38" s="52"/>
-      <c r="BV38" s="56"/>
-      <c r="BW38" s="56"/>
-      <c r="BX38" s="56"/>
-      <c r="BY38" s="56"/>
-      <c r="BZ38" s="56"/>
-      <c r="CA38" s="56"/>
+      <c r="BV38" s="55"/>
+      <c r="BW38" s="55"/>
+      <c r="BX38" s="55"/>
+      <c r="BY38" s="55"/>
+      <c r="BZ38" s="55"/>
+      <c r="CA38" s="55"/>
       <c r="CB38" s="52"/>
       <c r="CC38" s="52"/>
       <c r="CD38" s="52"/>
@@ -6195,12 +6251,12 @@
       <c r="BV39" s="52"/>
       <c r="BW39" s="52"/>
       <c r="BX39" s="52"/>
-      <c r="BY39" s="56"/>
-      <c r="BZ39" s="56"/>
-      <c r="CA39" s="56"/>
-      <c r="CB39" s="56"/>
-      <c r="CC39" s="56"/>
-      <c r="CD39" s="56"/>
+      <c r="BY39" s="55"/>
+      <c r="BZ39" s="55"/>
+      <c r="CA39" s="55"/>
+      <c r="CB39" s="55"/>
+      <c r="CC39" s="55"/>
+      <c r="CD39" s="55"/>
       <c r="CE39" s="52"/>
       <c r="CF39" s="52"/>
       <c r="CG39" s="52"/>
@@ -6328,12 +6384,12 @@
       <c r="BY40" s="52"/>
       <c r="BZ40" s="52"/>
       <c r="CA40" s="52"/>
-      <c r="CB40" s="56"/>
-      <c r="CC40" s="56"/>
-      <c r="CD40" s="56"/>
-      <c r="CE40" s="56"/>
-      <c r="CF40" s="56"/>
-      <c r="CG40" s="56"/>
+      <c r="CB40" s="55"/>
+      <c r="CC40" s="55"/>
+      <c r="CD40" s="55"/>
+      <c r="CE40" s="55"/>
+      <c r="CF40" s="55"/>
+      <c r="CG40" s="55"/>
       <c r="CH40" s="52"/>
       <c r="CI40" s="52"/>
       <c r="CJ40" s="52"/>
@@ -6457,13 +6513,13 @@
       <c r="BX41" s="52"/>
       <c r="BY41" s="52"/>
       <c r="BZ41" s="52"/>
-      <c r="CA41" s="56"/>
-      <c r="CB41" s="56"/>
-      <c r="CC41" s="56"/>
-      <c r="CD41" s="56"/>
-      <c r="CE41" s="56"/>
-      <c r="CF41" s="56"/>
-      <c r="CG41" s="56"/>
+      <c r="CA41" s="55"/>
+      <c r="CB41" s="55"/>
+      <c r="CC41" s="55"/>
+      <c r="CD41" s="55"/>
+      <c r="CE41" s="55"/>
+      <c r="CF41" s="55"/>
+      <c r="CG41" s="55"/>
       <c r="CH41" s="52"/>
       <c r="CI41" s="52"/>
       <c r="CJ41" s="52"/>
@@ -6502,10 +6558,18 @@
         <v>79</v>
       </c>
       <c r="D42" s="42"/>
-      <c r="E42" s="43"/>
-      <c r="F42" s="43"/>
-      <c r="G42" s="44"/>
-      <c r="H42" s="45"/>
+      <c r="E42" s="43">
+        <f>MIN(E43:E45)</f>
+      </c>
+      <c r="F42" s="43">
+        <f>MAX(F43:F45)</f>
+      </c>
+      <c r="G42" s="44">
+        <f>DAYS(F42,E42)+1</f>
+      </c>
+      <c r="H42" s="45">
+        <f>AVERAGE(H43:H45)</f>
+      </c>
       <c r="I42" s="46"/>
       <c r="J42" s="46"/>
       <c r="K42" s="46"/>
@@ -6705,12 +6769,12 @@
       <c r="BW43" s="52"/>
       <c r="BX43" s="52"/>
       <c r="BY43" s="52"/>
-      <c r="BZ43" s="56"/>
-      <c r="CA43" s="56"/>
-      <c r="CB43" s="56"/>
-      <c r="CC43" s="56"/>
-      <c r="CD43" s="56"/>
-      <c r="CE43" s="56"/>
+      <c r="BZ43" s="55"/>
+      <c r="CA43" s="55"/>
+      <c r="CB43" s="55"/>
+      <c r="CC43" s="55"/>
+      <c r="CD43" s="55"/>
+      <c r="CE43" s="55"/>
       <c r="CF43" s="52"/>
       <c r="CG43" s="52"/>
       <c r="CH43" s="52"/>
@@ -6838,11 +6902,11 @@
       <c r="BZ44" s="52"/>
       <c r="CA44" s="52"/>
       <c r="CB44" s="52"/>
-      <c r="CC44" s="56"/>
-      <c r="CD44" s="56"/>
-      <c r="CE44" s="56"/>
-      <c r="CF44" s="56"/>
-      <c r="CG44" s="56"/>
+      <c r="CC44" s="55"/>
+      <c r="CD44" s="55"/>
+      <c r="CE44" s="55"/>
+      <c r="CF44" s="55"/>
+      <c r="CG44" s="55"/>
       <c r="CH44" s="52"/>
       <c r="CI44" s="52"/>
       <c r="CJ44" s="52"/>
@@ -6881,7 +6945,7 @@
         <v>82</v>
       </c>
       <c r="D45" s="48" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E45" s="49">
         <v>46334</v>
@@ -6968,11 +7032,11 @@
       <c r="BZ45" s="52"/>
       <c r="CA45" s="52"/>
       <c r="CB45" s="52"/>
-      <c r="CC45" s="56"/>
-      <c r="CD45" s="56"/>
-      <c r="CE45" s="56"/>
-      <c r="CF45" s="56"/>
-      <c r="CG45" s="56"/>
+      <c r="CC45" s="55"/>
+      <c r="CD45" s="55"/>
+      <c r="CE45" s="55"/>
+      <c r="CF45" s="55"/>
+      <c r="CG45" s="55"/>
       <c r="CH45" s="52"/>
       <c r="CI45" s="52"/>
       <c r="CJ45" s="52"/>
@@ -7011,10 +7075,18 @@
         <v>83</v>
       </c>
       <c r="D46" s="42"/>
-      <c r="E46" s="43"/>
-      <c r="F46" s="43"/>
-      <c r="G46" s="44"/>
-      <c r="H46" s="45"/>
+      <c r="E46" s="43">
+        <f>MIN(E47:E50)</f>
+      </c>
+      <c r="F46" s="43">
+        <f>MAX(F47:F50)</f>
+      </c>
+      <c r="G46" s="44">
+        <f>DAYS(F46,E46)+1</f>
+      </c>
+      <c r="H46" s="45">
+        <f>AVERAGE(H47:H50)</f>
+      </c>
       <c r="I46" s="46"/>
       <c r="J46" s="46"/>
       <c r="K46" s="46"/>
@@ -7222,12 +7294,12 @@
       <c r="CE47" s="52"/>
       <c r="CF47" s="52"/>
       <c r="CG47" s="52"/>
-      <c r="CH47" s="57"/>
-      <c r="CI47" s="57"/>
-      <c r="CJ47" s="57"/>
-      <c r="CK47" s="57"/>
-      <c r="CL47" s="57"/>
-      <c r="CM47" s="57"/>
+      <c r="CH47" s="55"/>
+      <c r="CI47" s="55"/>
+      <c r="CJ47" s="55"/>
+      <c r="CK47" s="55"/>
+      <c r="CL47" s="55"/>
+      <c r="CM47" s="55"/>
       <c r="CN47" s="52"/>
       <c r="CO47" s="52"/>
       <c r="CP47" s="52"/>
@@ -7355,12 +7427,12 @@
       <c r="CH48" s="52"/>
       <c r="CI48" s="52"/>
       <c r="CJ48" s="52"/>
-      <c r="CK48" s="57"/>
-      <c r="CL48" s="57"/>
-      <c r="CM48" s="57"/>
-      <c r="CN48" s="57"/>
-      <c r="CO48" s="57"/>
-      <c r="CP48" s="57"/>
+      <c r="CK48" s="55"/>
+      <c r="CL48" s="55"/>
+      <c r="CM48" s="55"/>
+      <c r="CN48" s="55"/>
+      <c r="CO48" s="55"/>
+      <c r="CP48" s="55"/>
       <c r="CQ48" s="52"/>
       <c r="CR48" s="52"/>
       <c r="CS48" s="52"/>
@@ -7488,11 +7560,11 @@
       <c r="CK49" s="52"/>
       <c r="CL49" s="52"/>
       <c r="CM49" s="52"/>
-      <c r="CN49" s="57"/>
-      <c r="CO49" s="57"/>
-      <c r="CP49" s="57"/>
-      <c r="CQ49" s="57"/>
-      <c r="CR49" s="57"/>
+      <c r="CN49" s="55"/>
+      <c r="CO49" s="55"/>
+      <c r="CP49" s="55"/>
+      <c r="CQ49" s="55"/>
+      <c r="CR49" s="55"/>
       <c r="CS49" s="52"/>
       <c r="CT49" s="52"/>
       <c r="CU49" s="52"/>
@@ -7619,11 +7691,11 @@
       <c r="CL50" s="52"/>
       <c r="CM50" s="52"/>
       <c r="CN50" s="52"/>
-      <c r="CO50" s="57"/>
-      <c r="CP50" s="57"/>
-      <c r="CQ50" s="57"/>
-      <c r="CR50" s="57"/>
-      <c r="CS50" s="57"/>
+      <c r="CO50" s="55"/>
+      <c r="CP50" s="55"/>
+      <c r="CQ50" s="55"/>
+      <c r="CR50" s="55"/>
+      <c r="CS50" s="55"/>
       <c r="CT50" s="52"/>
       <c r="CU50" s="52"/>
       <c r="CV50" s="52"/>
@@ -7650,10 +7722,18 @@
         <v>88</v>
       </c>
       <c r="D51" s="42"/>
-      <c r="E51" s="43"/>
-      <c r="F51" s="43"/>
-      <c r="G51" s="44"/>
-      <c r="H51" s="45"/>
+      <c r="E51" s="43">
+        <f>MIN(E52:E54)</f>
+      </c>
+      <c r="F51" s="43">
+        <f>MAX(F52:F54)</f>
+      </c>
+      <c r="G51" s="44">
+        <f>DAYS(F51,E51)+1</f>
+      </c>
+      <c r="H51" s="45">
+        <f>AVERAGE(H52:H54)</f>
+      </c>
       <c r="I51" s="46"/>
       <c r="J51" s="46"/>
       <c r="K51" s="46"/>
@@ -7865,11 +7945,11 @@
       <c r="CI52" s="52"/>
       <c r="CJ52" s="52"/>
       <c r="CK52" s="52"/>
-      <c r="CL52" s="57"/>
-      <c r="CM52" s="57"/>
-      <c r="CN52" s="57"/>
-      <c r="CO52" s="57"/>
-      <c r="CP52" s="57"/>
+      <c r="CL52" s="55"/>
+      <c r="CM52" s="55"/>
+      <c r="CN52" s="55"/>
+      <c r="CO52" s="55"/>
+      <c r="CP52" s="55"/>
       <c r="CQ52" s="52"/>
       <c r="CR52" s="52"/>
       <c r="CS52" s="52"/>
@@ -7998,12 +8078,12 @@
       <c r="CL53" s="52"/>
       <c r="CM53" s="52"/>
       <c r="CN53" s="52"/>
-      <c r="CO53" s="57"/>
-      <c r="CP53" s="57"/>
-      <c r="CQ53" s="57"/>
-      <c r="CR53" s="57"/>
-      <c r="CS53" s="57"/>
-      <c r="CT53" s="57"/>
+      <c r="CO53" s="55"/>
+      <c r="CP53" s="55"/>
+      <c r="CQ53" s="55"/>
+      <c r="CR53" s="55"/>
+      <c r="CS53" s="55"/>
+      <c r="CT53" s="55"/>
       <c r="CU53" s="52"/>
       <c r="CV53" s="52"/>
       <c r="CW53" s="52"/>
@@ -8131,10 +8211,10 @@
       <c r="CO54" s="52"/>
       <c r="CP54" s="52"/>
       <c r="CQ54" s="52"/>
-      <c r="CR54" s="57"/>
-      <c r="CS54" s="57"/>
-      <c r="CT54" s="57"/>
-      <c r="CU54" s="57"/>
+      <c r="CR54" s="55"/>
+      <c r="CS54" s="55"/>
+      <c r="CT54" s="55"/>
+      <c r="CU54" s="55"/>
       <c r="CV54" s="52"/>
       <c r="CW54" s="52"/>
       <c r="CX54" s="52"/>
@@ -8159,10 +8239,18 @@
         <v>92</v>
       </c>
       <c r="D55" s="42"/>
-      <c r="E55" s="43"/>
-      <c r="F55" s="43"/>
-      <c r="G55" s="44"/>
-      <c r="H55" s="45"/>
+      <c r="E55" s="43">
+        <f>MIN(E56:E60)</f>
+      </c>
+      <c r="F55" s="43">
+        <f>MAX(F56:F60)</f>
+      </c>
+      <c r="G55" s="44">
+        <f>DAYS(F55,E55)+1</f>
+      </c>
+      <c r="H55" s="45">
+        <f>AVERAGE(H56:H60)</f>
+      </c>
       <c r="I55" s="46"/>
       <c r="J55" s="46"/>
       <c r="K55" s="46"/>
@@ -8384,11 +8472,11 @@
       <c r="CS56" s="52"/>
       <c r="CT56" s="52"/>
       <c r="CU56" s="52"/>
-      <c r="CV56" s="62"/>
-      <c r="CW56" s="62"/>
-      <c r="CX56" s="62"/>
-      <c r="CY56" s="62"/>
-      <c r="CZ56" s="62"/>
+      <c r="CV56" s="55"/>
+      <c r="CW56" s="55"/>
+      <c r="CX56" s="55"/>
+      <c r="CY56" s="55"/>
+      <c r="CZ56" s="55"/>
       <c r="DA56" s="52"/>
       <c r="DB56" s="52"/>
       <c r="DC56" s="52"/>
@@ -8516,12 +8604,12 @@
       <c r="CU57" s="52"/>
       <c r="CV57" s="52"/>
       <c r="CW57" s="52"/>
-      <c r="CX57" s="62"/>
-      <c r="CY57" s="62"/>
-      <c r="CZ57" s="62"/>
-      <c r="DA57" s="62"/>
-      <c r="DB57" s="62"/>
-      <c r="DC57" s="62"/>
+      <c r="CX57" s="55"/>
+      <c r="CY57" s="55"/>
+      <c r="CZ57" s="55"/>
+      <c r="DA57" s="55"/>
+      <c r="DB57" s="55"/>
+      <c r="DC57" s="55"/>
       <c r="DD57" s="52"/>
       <c r="DE57" s="52"/>
       <c r="DF57" s="52"/>
@@ -8648,12 +8736,12 @@
       <c r="CW58" s="52"/>
       <c r="CX58" s="52"/>
       <c r="CY58" s="52"/>
-      <c r="CZ58" s="62"/>
-      <c r="DA58" s="62"/>
-      <c r="DB58" s="62"/>
-      <c r="DC58" s="62"/>
-      <c r="DD58" s="62"/>
-      <c r="DE58" s="62"/>
+      <c r="CZ58" s="55"/>
+      <c r="DA58" s="55"/>
+      <c r="DB58" s="55"/>
+      <c r="DC58" s="55"/>
+      <c r="DD58" s="55"/>
+      <c r="DE58" s="55"/>
       <c r="DF58" s="52"/>
       <c r="DG58" s="52"/>
       <c r="DH58" s="52"/>
@@ -8780,11 +8868,11 @@
       <c r="CY59" s="52"/>
       <c r="CZ59" s="52"/>
       <c r="DA59" s="52"/>
-      <c r="DB59" s="62"/>
-      <c r="DC59" s="62"/>
-      <c r="DD59" s="62"/>
-      <c r="DE59" s="62"/>
-      <c r="DF59" s="62"/>
+      <c r="DB59" s="55"/>
+      <c r="DC59" s="55"/>
+      <c r="DD59" s="55"/>
+      <c r="DE59" s="55"/>
+      <c r="DF59" s="55"/>
       <c r="DG59" s="52"/>
       <c r="DH59" s="52"/>
       <c r="DI59" s="52"/>
@@ -8913,9 +9001,9 @@
       <c r="DB60" s="52"/>
       <c r="DC60" s="52"/>
       <c r="DD60" s="52"/>
-      <c r="DE60" s="62"/>
-      <c r="DF60" s="62"/>
-      <c r="DG60" s="62"/>
+      <c r="DE60" s="55"/>
+      <c r="DF60" s="55"/>
+      <c r="DG60" s="55"/>
       <c r="DH60" s="52"/>
       <c r="DI60" s="52"/>
     </row>
@@ -8928,10 +9016,18 @@
         <v>98</v>
       </c>
       <c r="D61" s="42"/>
-      <c r="E61" s="43"/>
-      <c r="F61" s="43"/>
-      <c r="G61" s="44"/>
-      <c r="H61" s="45"/>
+      <c r="E61" s="43">
+        <f>MIN(E62:E65)</f>
+      </c>
+      <c r="F61" s="43">
+        <f>MAX(F62:F65)</f>
+      </c>
+      <c r="G61" s="44">
+        <f>DAYS(F61,E61)+1</f>
+      </c>
+      <c r="H61" s="45">
+        <f>AVERAGE(H62:H65)</f>
+      </c>
       <c r="I61" s="46"/>
       <c r="J61" s="46"/>
       <c r="K61" s="46"/>
@@ -9160,11 +9256,11 @@
       <c r="CZ62" s="52"/>
       <c r="DA62" s="52"/>
       <c r="DB62" s="52"/>
-      <c r="DC62" s="62"/>
-      <c r="DD62" s="62"/>
-      <c r="DE62" s="62"/>
-      <c r="DF62" s="62"/>
-      <c r="DG62" s="62"/>
+      <c r="DC62" s="55"/>
+      <c r="DD62" s="55"/>
+      <c r="DE62" s="55"/>
+      <c r="DF62" s="55"/>
+      <c r="DG62" s="55"/>
       <c r="DH62" s="52"/>
       <c r="DI62" s="52"/>
     </row>
@@ -9293,9 +9389,9 @@
       <c r="DC63" s="52"/>
       <c r="DD63" s="52"/>
       <c r="DE63" s="52"/>
-      <c r="DF63" s="62"/>
-      <c r="DG63" s="62"/>
-      <c r="DH63" s="62"/>
+      <c r="DF63" s="55"/>
+      <c r="DG63" s="55"/>
+      <c r="DH63" s="55"/>
       <c r="DI63" s="52"/>
     </row>
     <row r="64" ht="18.0" customHeight="1">
@@ -9424,8 +9520,8 @@
       <c r="DD64" s="52"/>
       <c r="DE64" s="52"/>
       <c r="DF64" s="52"/>
-      <c r="DG64" s="62"/>
-      <c r="DH64" s="62"/>
+      <c r="DG64" s="55"/>
+      <c r="DH64" s="55"/>
       <c r="DI64" s="52"/>
     </row>
     <row r="65" ht="18.0" customHeight="1">
@@ -9556,7 +9652,7 @@
       <c r="DF65" s="52"/>
       <c r="DG65" s="52"/>
       <c r="DH65" s="52"/>
-      <c r="DI65" s="62"/>
+      <c r="DI65" s="55"/>
     </row>
     <row r="66" ht="18.0" customHeight="1">
       <c r="A66" s="4"/>

</xml_diff>